<commit_message>
update Diagrama de Gantt
</commit_message>
<xml_diff>
--- a/Diagrama de Gantt.xlsx
+++ b/Diagrama de Gantt.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\df335\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\df335\Desktop\ProyectoFinDeCursoGrupo5\ProyectoFinDeCursoGrupo5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B91ED9EC-D1FD-4E10-AEA9-DA74398BE995}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52517594-123F-4E85-90C9-16056C31DD7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{75261B6F-E73A-4DEC-92A2-DFBB6B85624B}"/>
   </bookViews>
@@ -166,7 +166,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -183,6 +183,14 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -306,7 +314,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -335,6 +343,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -649,10 +658,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{014F5967-FF16-4A7A-8914-B6A3D6DBE291}">
-  <dimension ref="A3:AJ13"/>
+  <dimension ref="A3:AJ34"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.109375" customWidth="1"/>
+    <col min="1" max="1" width="16.109375" customWidth="1"/>
     <col min="2" max="2" width="13.6640625" customWidth="1"/>
     <col min="3" max="3" width="13.44140625" customWidth="1"/>
     <col min="4" max="4" width="13.88671875" customWidth="1"/>
@@ -975,8 +984,12 @@
         <v>0</v>
       </c>
     </row>
+    <row r="34" spans="9:9" x14ac:dyDescent="0.3">
+      <c r="I34" s="14"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>